<commit_message>
Scan index: mycotoxins of the sent CoQs -085 and -131, read off their scans (all ND from Farmahem, no n/t cell)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01DyBhj47i7bhaCyNMB1iwdv
</commit_message>
<xml_diff>
--- a/deliverables/qc_gap_analysis/tracker/SCAN_INDEX_2026-09-25.xlsx
+++ b/deliverables/qc_gap_analysis/tracker/SCAN_INDEX_2026-09-25.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Approved scans" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Approved scans'!$A$1:$Z$47</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Approved scans'!$A$1:$AE$47</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -458,7 +458,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z47"/>
+  <dimension ref="A1:AE47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -483,10 +483,15 @@
     <col width="9" customWidth="1" min="20" max="20"/>
     <col width="9" customWidth="1" min="21" max="21"/>
     <col width="9" customWidth="1" min="22" max="22"/>
-    <col width="36" customWidth="1" min="23" max="23"/>
-    <col width="20" customWidth="1" min="24" max="24"/>
-    <col width="11" customWidth="1" min="25" max="25"/>
-    <col width="34" customWidth="1" min="26" max="26"/>
+    <col width="9" customWidth="1" min="23" max="23"/>
+    <col width="9" customWidth="1" min="24" max="24"/>
+    <col width="9" customWidth="1" min="25" max="25"/>
+    <col width="9" customWidth="1" min="26" max="26"/>
+    <col width="9" customWidth="1" min="27" max="27"/>
+    <col width="36" customWidth="1" min="28" max="28"/>
+    <col width="20" customWidth="1" min="29" max="29"/>
+    <col width="11" customWidth="1" min="30" max="30"/>
+    <col width="34" customWidth="1" min="31" max="31"/>
   </cols>
   <sheetData>
     <row r="1" ht="42" customHeight="1">
@@ -602,20 +607,45 @@
       </c>
       <c r="W1" s="1" t="inlineStr">
         <is>
+          <t>B1</t>
+        </is>
+      </c>
+      <c r="X1" s="1" t="inlineStr">
+        <is>
+          <t>aflatoxins_total</t>
+        </is>
+      </c>
+      <c r="Y1" s="1" t="inlineStr">
+        <is>
+          <t>OTA</t>
+        </is>
+      </c>
+      <c r="Z1" s="1" t="inlineStr">
+        <is>
+          <t>mycotoxin_cert</t>
+        </is>
+      </c>
+      <c r="AA1" s="1" t="inlineStr">
+        <is>
+          <t>not_tested_cells</t>
+        </is>
+      </c>
+      <c r="AB1" s="1" t="inlineStr">
+        <is>
           <t>drive_file_id</t>
         </is>
       </c>
-      <c r="X1" s="1" t="inlineStr">
+      <c r="AC1" s="1" t="inlineStr">
         <is>
           <t>drive_title</t>
         </is>
       </c>
-      <c r="Y1" s="1" t="inlineStr">
+      <c r="AD1" s="1" t="inlineStr">
         <is>
           <t>drive_bytes</t>
         </is>
       </c>
-      <c r="Z1" s="1" t="inlineStr">
+      <c r="AE1" s="1" t="inlineStr">
         <is>
           <t>note</t>
         </is>
@@ -728,22 +758,47 @@
           <t>0.005</t>
         </is>
       </c>
-      <c r="W2" s="5" t="inlineStr">
+      <c r="W2" s="2" t="inlineStr">
+        <is>
+          <t>ND</t>
+        </is>
+      </c>
+      <c r="X2" s="2" t="inlineStr">
+        <is>
+          <t>ND</t>
+        </is>
+      </c>
+      <c r="Y2" s="2" t="inlineStr">
+        <is>
+          <t>ND</t>
+        </is>
+      </c>
+      <c r="Z2" s="2" t="inlineStr">
+        <is>
+          <t>197-1-М/26 (10.08.2026)</t>
+        </is>
+      </c>
+      <c r="AA2" s="2" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="AB2" s="5" t="inlineStr">
         <is>
           <t>1mYg_gnva5q9K_-uTY2MPIN46iq8aMebC</t>
         </is>
       </c>
-      <c r="X2" s="5" t="inlineStr">
+      <c r="AC2" s="5" t="inlineStr">
         <is>
           <t>BG1024 (1).pdf</t>
         </is>
       </c>
-      <c r="Y2" s="5" t="inlineStr">
+      <c r="AD2" s="5" t="inlineStr">
         <is>
           <t>525357</t>
         </is>
       </c>
-      <c r="Z2" s="2" t="inlineStr"/>
+      <c r="AE2" s="2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -852,22 +907,27 @@
           <t>0.014</t>
         </is>
       </c>
-      <c r="W3" s="5" t="inlineStr">
+      <c r="W3" s="2" t="inlineStr"/>
+      <c r="X3" s="2" t="inlineStr"/>
+      <c r="Y3" s="2" t="inlineStr"/>
+      <c r="Z3" s="2" t="inlineStr"/>
+      <c r="AA3" s="2" t="inlineStr"/>
+      <c r="AB3" s="5" t="inlineStr">
         <is>
           <t>1turLjlkueTZLO_wWRfUw-eqJuxJQ8hmq</t>
         </is>
       </c>
-      <c r="X3" s="5" t="inlineStr">
+      <c r="AC3" s="5" t="inlineStr">
         <is>
           <t>BSS1024 (1).pdf</t>
         </is>
       </c>
-      <c r="Y3" s="5" t="inlineStr">
+      <c r="AD3" s="5" t="inlineStr">
         <is>
           <t>537588</t>
         </is>
       </c>
-      <c r="Z3" s="2" t="inlineStr"/>
+      <c r="AE3" s="2" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -976,22 +1036,27 @@
           <t>0.004</t>
         </is>
       </c>
-      <c r="W4" s="5" t="inlineStr">
+      <c r="W4" s="2" t="inlineStr"/>
+      <c r="X4" s="2" t="inlineStr"/>
+      <c r="Y4" s="2" t="inlineStr"/>
+      <c r="Z4" s="2" t="inlineStr"/>
+      <c r="AA4" s="2" t="inlineStr"/>
+      <c r="AB4" s="5" t="inlineStr">
         <is>
           <t>1wFgq1tRmzVzzce4TGeqytI5zEU7j19sA</t>
         </is>
       </c>
-      <c r="X4" s="5" t="inlineStr">
+      <c r="AC4" s="5" t="inlineStr">
         <is>
           <t>GG1024.pdf</t>
         </is>
       </c>
-      <c r="Y4" s="5" t="inlineStr">
+      <c r="AD4" s="5" t="inlineStr">
         <is>
           <t>552729</t>
         </is>
       </c>
-      <c r="Z4" s="2" t="inlineStr"/>
+      <c r="AE4" s="2" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -1100,22 +1165,27 @@
           <t>0.005</t>
         </is>
       </c>
-      <c r="W5" s="5" t="inlineStr">
+      <c r="W5" s="2" t="inlineStr"/>
+      <c r="X5" s="2" t="inlineStr"/>
+      <c r="Y5" s="2" t="inlineStr"/>
+      <c r="Z5" s="2" t="inlineStr"/>
+      <c r="AA5" s="2" t="inlineStr"/>
+      <c r="AB5" s="5" t="inlineStr">
         <is>
           <t>1JfttSl_EiBYPHn7KXwUZDu3GpcnaGFJ8</t>
         </is>
       </c>
-      <c r="X5" s="5" t="inlineStr">
+      <c r="AC5" s="5" t="inlineStr">
         <is>
           <t>HPA1024 (1).pdf</t>
         </is>
       </c>
-      <c r="Y5" s="5" t="inlineStr">
+      <c r="AD5" s="5" t="inlineStr">
         <is>
           <t>586000</t>
         </is>
       </c>
-      <c r="Z5" s="2" t="inlineStr"/>
+      <c r="AE5" s="2" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -1224,22 +1294,27 @@
           <t>0.005</t>
         </is>
       </c>
-      <c r="W6" s="5" t="inlineStr">
+      <c r="W6" s="2" t="inlineStr"/>
+      <c r="X6" s="2" t="inlineStr"/>
+      <c r="Y6" s="2" t="inlineStr"/>
+      <c r="Z6" s="2" t="inlineStr"/>
+      <c r="AA6" s="2" t="inlineStr"/>
+      <c r="AB6" s="5" t="inlineStr">
         <is>
           <t>197eKpSvdDzUReYy4AMXZxuhxeKwD7mNW</t>
         </is>
       </c>
-      <c r="X6" s="5" t="inlineStr">
+      <c r="AC6" s="5" t="inlineStr">
         <is>
           <t>OPM1024 (2).pdf</t>
         </is>
       </c>
-      <c r="Y6" s="5" t="inlineStr">
+      <c r="AD6" s="5" t="inlineStr">
         <is>
           <t>602406</t>
         </is>
       </c>
-      <c r="Z6" s="2" t="inlineStr"/>
+      <c r="AE6" s="2" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -1348,22 +1423,27 @@
           <t>ND</t>
         </is>
       </c>
-      <c r="W7" s="5" t="inlineStr">
+      <c r="W7" s="2" t="inlineStr"/>
+      <c r="X7" s="2" t="inlineStr"/>
+      <c r="Y7" s="2" t="inlineStr"/>
+      <c r="Z7" s="2" t="inlineStr"/>
+      <c r="AA7" s="2" t="inlineStr"/>
+      <c r="AB7" s="5" t="inlineStr">
         <is>
           <t>1zohLeaQP8EoB5RHusPhsc3yqDg0Ut2YS</t>
         </is>
       </c>
-      <c r="X7" s="5" t="inlineStr">
+      <c r="AC7" s="5" t="inlineStr">
         <is>
           <t>P05022 (1).pdf</t>
         </is>
       </c>
-      <c r="Y7" s="5" t="inlineStr">
+      <c r="AD7" s="5" t="inlineStr">
         <is>
           <t>525138</t>
         </is>
       </c>
-      <c r="Z7" s="2" t="inlineStr"/>
+      <c r="AE7" s="2" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -1472,22 +1552,27 @@
           <t>0.001</t>
         </is>
       </c>
-      <c r="W8" s="5" t="inlineStr">
+      <c r="W8" s="2" t="inlineStr"/>
+      <c r="X8" s="2" t="inlineStr"/>
+      <c r="Y8" s="2" t="inlineStr"/>
+      <c r="Z8" s="2" t="inlineStr"/>
+      <c r="AA8" s="2" t="inlineStr"/>
+      <c r="AB8" s="5" t="inlineStr">
         <is>
           <t>1160fGfnTKso4Lf99QI0WYpVRS-K1CHD3</t>
         </is>
       </c>
-      <c r="X8" s="5" t="inlineStr">
+      <c r="AC8" s="5" t="inlineStr">
         <is>
           <t>P050042.pdf</t>
         </is>
       </c>
-      <c r="Y8" s="5" t="inlineStr">
+      <c r="AD8" s="5" t="inlineStr">
         <is>
           <t>545409</t>
         </is>
       </c>
-      <c r="Z8" s="2" t="inlineStr"/>
+      <c r="AE8" s="2" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -1596,22 +1681,27 @@
           <t>0.008</t>
         </is>
       </c>
-      <c r="W9" s="5" t="inlineStr">
+      <c r="W9" s="2" t="inlineStr"/>
+      <c r="X9" s="2" t="inlineStr"/>
+      <c r="Y9" s="2" t="inlineStr"/>
+      <c r="Z9" s="2" t="inlineStr"/>
+      <c r="AA9" s="2" t="inlineStr"/>
+      <c r="AB9" s="5" t="inlineStr">
         <is>
           <t>1aNIH7twrFoPI0z6tRErQ6TPp9vSAJKu7</t>
         </is>
       </c>
-      <c r="X9" s="5" t="inlineStr">
+      <c r="AC9" s="5" t="inlineStr">
         <is>
           <t>P050052 (1).pdf</t>
         </is>
       </c>
-      <c r="Y9" s="5" t="inlineStr">
+      <c r="AD9" s="5" t="inlineStr">
         <is>
           <t>527165</t>
         </is>
       </c>
-      <c r="Z9" s="2" t="inlineStr"/>
+      <c r="AE9" s="2" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -1720,22 +1810,27 @@
           <t>0.061</t>
         </is>
       </c>
-      <c r="W10" s="5" t="inlineStr">
+      <c r="W10" s="2" t="inlineStr"/>
+      <c r="X10" s="2" t="inlineStr"/>
+      <c r="Y10" s="2" t="inlineStr"/>
+      <c r="Z10" s="2" t="inlineStr"/>
+      <c r="AA10" s="2" t="inlineStr"/>
+      <c r="AB10" s="5" t="inlineStr">
         <is>
           <t>1AJOSv6xceSgU-vVhP9mxRLMc9j4sPdh0</t>
         </is>
       </c>
-      <c r="X10" s="5" t="inlineStr">
+      <c r="AC10" s="5" t="inlineStr">
         <is>
           <t>P050062 (1).pdf</t>
         </is>
       </c>
-      <c r="Y10" s="5" t="inlineStr">
+      <c r="AD10" s="5" t="inlineStr">
         <is>
           <t>533133</t>
         </is>
       </c>
-      <c r="Z10" s="2" t="inlineStr"/>
+      <c r="AE10" s="2" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -1844,22 +1939,27 @@
           <t>ND</t>
         </is>
       </c>
-      <c r="W11" s="5" t="inlineStr">
+      <c r="W11" s="2" t="inlineStr"/>
+      <c r="X11" s="2" t="inlineStr"/>
+      <c r="Y11" s="2" t="inlineStr"/>
+      <c r="Z11" s="2" t="inlineStr"/>
+      <c r="AA11" s="2" t="inlineStr"/>
+      <c r="AB11" s="5" t="inlineStr">
         <is>
           <t>11nlikkWSKe7IQQb7QiTXhaJ7hn7GQJJy</t>
         </is>
       </c>
-      <c r="X11" s="5" t="inlineStr">
+      <c r="AC11" s="5" t="inlineStr">
         <is>
           <t>P050072.pdf</t>
         </is>
       </c>
-      <c r="Y11" s="5" t="inlineStr">
+      <c r="AD11" s="5" t="inlineStr">
         <is>
           <t>557170</t>
         </is>
       </c>
-      <c r="Z11" s="2" t="inlineStr"/>
+      <c r="AE11" s="2" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -1968,22 +2068,27 @@
           <t>0.03</t>
         </is>
       </c>
-      <c r="W12" s="5" t="inlineStr">
+      <c r="W12" s="2" t="inlineStr"/>
+      <c r="X12" s="2" t="inlineStr"/>
+      <c r="Y12" s="2" t="inlineStr"/>
+      <c r="Z12" s="2" t="inlineStr"/>
+      <c r="AA12" s="2" t="inlineStr"/>
+      <c r="AB12" s="5" t="inlineStr">
         <is>
           <t>1BkRyXlfNSKAcmInu6SLa3ieTUwZ_HnrM</t>
         </is>
       </c>
-      <c r="X12" s="5" t="inlineStr">
+      <c r="AC12" s="5" t="inlineStr">
         <is>
           <t>P050082.pdf</t>
         </is>
       </c>
-      <c r="Y12" s="5" t="inlineStr">
+      <c r="AD12" s="5" t="inlineStr">
         <is>
           <t>564220</t>
         </is>
       </c>
-      <c r="Z12" s="2" t="inlineStr"/>
+      <c r="AE12" s="2" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -2092,22 +2197,27 @@
           <t>0.005</t>
         </is>
       </c>
-      <c r="W13" s="5" t="inlineStr">
+      <c r="W13" s="2" t="inlineStr"/>
+      <c r="X13" s="2" t="inlineStr"/>
+      <c r="Y13" s="2" t="inlineStr"/>
+      <c r="Z13" s="2" t="inlineStr"/>
+      <c r="AA13" s="2" t="inlineStr"/>
+      <c r="AB13" s="5" t="inlineStr">
         <is>
           <t>1AC1woVYClWr7d8WNq4h-CdVhj6WtvFay</t>
         </is>
       </c>
-      <c r="X13" s="5" t="inlineStr">
+      <c r="AC13" s="5" t="inlineStr">
         <is>
           <t>P050092 (1).pdf</t>
         </is>
       </c>
-      <c r="Y13" s="5" t="inlineStr">
+      <c r="AD13" s="5" t="inlineStr">
         <is>
           <t>533113</t>
         </is>
       </c>
-      <c r="Z13" s="2" t="inlineStr"/>
+      <c r="AE13" s="2" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -2216,22 +2326,27 @@
           <t>0.006</t>
         </is>
       </c>
-      <c r="W14" s="5" t="inlineStr">
+      <c r="W14" s="2" t="inlineStr"/>
+      <c r="X14" s="2" t="inlineStr"/>
+      <c r="Y14" s="2" t="inlineStr"/>
+      <c r="Z14" s="2" t="inlineStr"/>
+      <c r="AA14" s="2" t="inlineStr"/>
+      <c r="AB14" s="5" t="inlineStr">
         <is>
           <t>1RDpsc6Cxe6tjff3DiAQJ3RzAEjgwIZjj</t>
         </is>
       </c>
-      <c r="X14" s="5" t="inlineStr">
+      <c r="AC14" s="5" t="inlineStr">
         <is>
           <t>P050112.pdf</t>
         </is>
       </c>
-      <c r="Y14" s="5" t="inlineStr">
+      <c r="AD14" s="5" t="inlineStr">
         <is>
           <t>516468</t>
         </is>
       </c>
-      <c r="Z14" s="2" t="inlineStr"/>
+      <c r="AE14" s="2" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -2340,22 +2455,27 @@
           <t>ND</t>
         </is>
       </c>
-      <c r="W15" s="5" t="inlineStr">
+      <c r="W15" s="2" t="inlineStr"/>
+      <c r="X15" s="2" t="inlineStr"/>
+      <c r="Y15" s="2" t="inlineStr"/>
+      <c r="Z15" s="2" t="inlineStr"/>
+      <c r="AA15" s="2" t="inlineStr"/>
+      <c r="AB15" s="5" t="inlineStr">
         <is>
           <t>1zncyh33vK0QsUBiegJhY60Coi27b1cuL</t>
         </is>
       </c>
-      <c r="X15" s="5" t="inlineStr">
+      <c r="AC15" s="5" t="inlineStr">
         <is>
           <t>P050152 (1).pdf</t>
         </is>
       </c>
-      <c r="Y15" s="5" t="inlineStr">
+      <c r="AD15" s="5" t="inlineStr">
         <is>
           <t>599894</t>
         </is>
       </c>
-      <c r="Z15" s="2" t="inlineStr"/>
+      <c r="AE15" s="2" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -2468,22 +2588,27 @@
           <t>ND</t>
         </is>
       </c>
-      <c r="W16" s="5" t="inlineStr">
+      <c r="W16" s="2" t="inlineStr"/>
+      <c r="X16" s="2" t="inlineStr"/>
+      <c r="Y16" s="2" t="inlineStr"/>
+      <c r="Z16" s="2" t="inlineStr"/>
+      <c r="AA16" s="2" t="inlineStr"/>
+      <c r="AB16" s="5" t="inlineStr">
         <is>
           <t>1GoAjyZUmajiBPUvVD00_5d8NGlVfImiP</t>
         </is>
       </c>
-      <c r="X16" s="5" t="inlineStr">
+      <c r="AC16" s="5" t="inlineStr">
         <is>
           <t>P050162 (1).pdf</t>
         </is>
       </c>
-      <c r="Y16" s="5" t="inlineStr">
+      <c r="AD16" s="5" t="inlineStr">
         <is>
           <t>532001</t>
         </is>
       </c>
-      <c r="Z16" s="2" t="inlineStr"/>
+      <c r="AE16" s="2" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -2592,22 +2717,27 @@
           <t>ND</t>
         </is>
       </c>
-      <c r="W17" s="5" t="inlineStr">
+      <c r="W17" s="2" t="inlineStr"/>
+      <c r="X17" s="2" t="inlineStr"/>
+      <c r="Y17" s="2" t="inlineStr"/>
+      <c r="Z17" s="2" t="inlineStr"/>
+      <c r="AA17" s="2" t="inlineStr"/>
+      <c r="AB17" s="5" t="inlineStr">
         <is>
           <t>1AcMuqofKNibr8-TN9T1-kk-cYNY8e5kx</t>
         </is>
       </c>
-      <c r="X17" s="5" t="inlineStr">
+      <c r="AC17" s="5" t="inlineStr">
         <is>
           <t>P050182.pdf</t>
         </is>
       </c>
-      <c r="Y17" s="5" t="inlineStr">
+      <c r="AD17" s="5" t="inlineStr">
         <is>
           <t>548582</t>
         </is>
       </c>
-      <c r="Z17" s="2" t="inlineStr"/>
+      <c r="AE17" s="2" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -2716,22 +2846,27 @@
           <t>0.0036</t>
         </is>
       </c>
-      <c r="W18" s="5" t="inlineStr">
+      <c r="W18" s="2" t="inlineStr"/>
+      <c r="X18" s="2" t="inlineStr"/>
+      <c r="Y18" s="2" t="inlineStr"/>
+      <c r="Z18" s="2" t="inlineStr"/>
+      <c r="AA18" s="2" t="inlineStr"/>
+      <c r="AB18" s="5" t="inlineStr">
         <is>
           <t>1uYZVOJh5teg0CpGKzG6V-Xdy_fNrhpVv</t>
         </is>
       </c>
-      <c r="X18" s="5" t="inlineStr">
+      <c r="AC18" s="5" t="inlineStr">
         <is>
           <t>P050192.pdf</t>
         </is>
       </c>
-      <c r="Y18" s="5" t="inlineStr">
+      <c r="AD18" s="5" t="inlineStr">
         <is>
           <t>558935</t>
         </is>
       </c>
-      <c r="Z18" s="2" t="inlineStr"/>
+      <c r="AE18" s="2" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -2844,22 +2979,27 @@
           <t>0.012</t>
         </is>
       </c>
-      <c r="W19" s="5" t="inlineStr">
+      <c r="W19" s="2" t="inlineStr"/>
+      <c r="X19" s="2" t="inlineStr"/>
+      <c r="Y19" s="2" t="inlineStr"/>
+      <c r="Z19" s="2" t="inlineStr"/>
+      <c r="AA19" s="2" t="inlineStr"/>
+      <c r="AB19" s="5" t="inlineStr">
         <is>
           <t>1X_ti3CJU5hY-7rKKD22emW0K4ToC0xHt</t>
         </is>
       </c>
-      <c r="X19" s="5" t="inlineStr">
+      <c r="AC19" s="5" t="inlineStr">
         <is>
           <t>P050212 (1).pdf</t>
         </is>
       </c>
-      <c r="Y19" s="5" t="inlineStr">
+      <c r="AD19" s="5" t="inlineStr">
         <is>
           <t>587576</t>
         </is>
       </c>
-      <c r="Z19" s="2" t="inlineStr"/>
+      <c r="AE19" s="2" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -2972,22 +3112,27 @@
           <t>0.017</t>
         </is>
       </c>
-      <c r="W20" s="5" t="inlineStr">
+      <c r="W20" s="2" t="inlineStr"/>
+      <c r="X20" s="2" t="inlineStr"/>
+      <c r="Y20" s="2" t="inlineStr"/>
+      <c r="Z20" s="2" t="inlineStr"/>
+      <c r="AA20" s="2" t="inlineStr"/>
+      <c r="AB20" s="5" t="inlineStr">
         <is>
           <t>1LYxCfQj4ZU22-vFn5fjjn76GID5y6X89</t>
         </is>
       </c>
-      <c r="X20" s="5" t="inlineStr">
+      <c r="AC20" s="5" t="inlineStr">
         <is>
           <t>P050222.pdf</t>
         </is>
       </c>
-      <c r="Y20" s="5" t="inlineStr">
+      <c r="AD20" s="5" t="inlineStr">
         <is>
           <t>557549</t>
         </is>
       </c>
-      <c r="Z20" s="2" t="inlineStr"/>
+      <c r="AE20" s="2" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -3096,22 +3241,27 @@
           <t>0.019</t>
         </is>
       </c>
-      <c r="W21" s="5" t="inlineStr">
+      <c r="W21" s="2" t="inlineStr"/>
+      <c r="X21" s="2" t="inlineStr"/>
+      <c r="Y21" s="2" t="inlineStr"/>
+      <c r="Z21" s="2" t="inlineStr"/>
+      <c r="AA21" s="2" t="inlineStr"/>
+      <c r="AB21" s="5" t="inlineStr">
         <is>
           <t>12RXpGLcUjqJZJFp1OOHSb0RcUevues4-</t>
         </is>
       </c>
-      <c r="X21" s="5" t="inlineStr">
+      <c r="AC21" s="5" t="inlineStr">
         <is>
           <t>P050302.pdf</t>
         </is>
       </c>
-      <c r="Y21" s="5" t="inlineStr">
+      <c r="AD21" s="5" t="inlineStr">
         <is>
           <t>551511</t>
         </is>
       </c>
-      <c r="Z21" s="2" t="inlineStr"/>
+      <c r="AE21" s="2" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -3220,22 +3370,27 @@
           <t>0.017</t>
         </is>
       </c>
-      <c r="W22" s="5" t="inlineStr">
+      <c r="W22" s="2" t="inlineStr"/>
+      <c r="X22" s="2" t="inlineStr"/>
+      <c r="Y22" s="2" t="inlineStr"/>
+      <c r="Z22" s="2" t="inlineStr"/>
+      <c r="AA22" s="2" t="inlineStr"/>
+      <c r="AB22" s="5" t="inlineStr">
         <is>
           <t>1_RXr492-uTsNrloa2HV8j3UTWCafT_mw</t>
         </is>
       </c>
-      <c r="X22" s="5" t="inlineStr">
+      <c r="AC22" s="5" t="inlineStr">
         <is>
           <t>P050312.pdf</t>
         </is>
       </c>
-      <c r="Y22" s="5" t="inlineStr">
+      <c r="AD22" s="5" t="inlineStr">
         <is>
           <t>554182</t>
         </is>
       </c>
-      <c r="Z22" s="2" t="inlineStr"/>
+      <c r="AE22" s="2" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -3344,22 +3499,27 @@
           <t>0.016</t>
         </is>
       </c>
-      <c r="W23" s="5" t="inlineStr">
+      <c r="W23" s="2" t="inlineStr"/>
+      <c r="X23" s="2" t="inlineStr"/>
+      <c r="Y23" s="2" t="inlineStr"/>
+      <c r="Z23" s="2" t="inlineStr"/>
+      <c r="AA23" s="2" t="inlineStr"/>
+      <c r="AB23" s="5" t="inlineStr">
         <is>
           <t>1RLjv9dih9XdRyOXsnIZEAwxbnuUBQnlz</t>
         </is>
       </c>
-      <c r="X23" s="5" t="inlineStr">
+      <c r="AC23" s="5" t="inlineStr">
         <is>
           <t>P050322 (1).pdf</t>
         </is>
       </c>
-      <c r="Y23" s="5" t="inlineStr">
+      <c r="AD23" s="5" t="inlineStr">
         <is>
           <t>526234</t>
         </is>
       </c>
-      <c r="Z23" s="2" t="inlineStr"/>
+      <c r="AE23" s="2" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -3468,22 +3628,27 @@
           <t>ND</t>
         </is>
       </c>
-      <c r="W24" s="5" t="inlineStr">
+      <c r="W24" s="2" t="inlineStr"/>
+      <c r="X24" s="2" t="inlineStr"/>
+      <c r="Y24" s="2" t="inlineStr"/>
+      <c r="Z24" s="2" t="inlineStr"/>
+      <c r="AA24" s="2" t="inlineStr"/>
+      <c r="AB24" s="5" t="inlineStr">
         <is>
           <t>1YZWBfZsgSGFztbLMWO1HfmPQTlhO88SL</t>
         </is>
       </c>
-      <c r="X24" s="5" t="inlineStr">
+      <c r="AC24" s="5" t="inlineStr">
         <is>
           <t>P060012.pdf</t>
         </is>
       </c>
-      <c r="Y24" s="5" t="inlineStr">
+      <c r="AD24" s="5" t="inlineStr">
         <is>
           <t>532565</t>
         </is>
       </c>
-      <c r="Z24" s="2" t="inlineStr"/>
+      <c r="AE24" s="2" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -3596,22 +3761,27 @@
           <t>ND</t>
         </is>
       </c>
-      <c r="W25" s="5" t="inlineStr">
+      <c r="W25" s="2" t="inlineStr"/>
+      <c r="X25" s="2" t="inlineStr"/>
+      <c r="Y25" s="2" t="inlineStr"/>
+      <c r="Z25" s="2" t="inlineStr"/>
+      <c r="AA25" s="2" t="inlineStr"/>
+      <c r="AB25" s="5" t="inlineStr">
         <is>
           <t>1QvRfshTmB8cwJ-tKSX6joVqo-zP5rD7N</t>
         </is>
       </c>
-      <c r="X25" s="5" t="inlineStr">
+      <c r="AC25" s="5" t="inlineStr">
         <is>
           <t>P060022.pdf</t>
         </is>
       </c>
-      <c r="Y25" s="5" t="inlineStr">
+      <c r="AD25" s="5" t="inlineStr">
         <is>
           <t>552250</t>
         </is>
       </c>
-      <c r="Z25" s="2" t="inlineStr"/>
+      <c r="AE25" s="2" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -3724,22 +3894,27 @@
           <t>ND</t>
         </is>
       </c>
-      <c r="W26" s="5" t="inlineStr">
+      <c r="W26" s="2" t="inlineStr"/>
+      <c r="X26" s="2" t="inlineStr"/>
+      <c r="Y26" s="2" t="inlineStr"/>
+      <c r="Z26" s="2" t="inlineStr"/>
+      <c r="AA26" s="2" t="inlineStr"/>
+      <c r="AB26" s="5" t="inlineStr">
         <is>
           <t>11TZRTwBsCCCfXNtgsokSj8HdtD99gU9C</t>
         </is>
       </c>
-      <c r="X26" s="5" t="inlineStr">
+      <c r="AC26" s="5" t="inlineStr">
         <is>
           <t>P060032 (1).pdf</t>
         </is>
       </c>
-      <c r="Y26" s="5" t="inlineStr">
+      <c r="AD26" s="5" t="inlineStr">
         <is>
           <t>529490</t>
         </is>
       </c>
-      <c r="Z26" s="2" t="inlineStr"/>
+      <c r="AE26" s="2" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
@@ -3848,22 +4023,27 @@
           <t>ND</t>
         </is>
       </c>
-      <c r="W27" s="5" t="inlineStr">
+      <c r="W27" s="2" t="inlineStr"/>
+      <c r="X27" s="2" t="inlineStr"/>
+      <c r="Y27" s="2" t="inlineStr"/>
+      <c r="Z27" s="2" t="inlineStr"/>
+      <c r="AA27" s="2" t="inlineStr"/>
+      <c r="AB27" s="5" t="inlineStr">
         <is>
           <t>1beEdBNg7cmEDeGFwhxKvJEu6qhk54i_M</t>
         </is>
       </c>
-      <c r="X27" s="5" t="inlineStr">
+      <c r="AC27" s="5" t="inlineStr">
         <is>
           <t>P060062 (1).pdf</t>
         </is>
       </c>
-      <c r="Y27" s="5" t="inlineStr">
+      <c r="AD27" s="5" t="inlineStr">
         <is>
           <t>533114</t>
         </is>
       </c>
-      <c r="Z27" s="2" t="inlineStr"/>
+      <c r="AE27" s="2" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -3976,22 +4156,27 @@
           <t>0.004</t>
         </is>
       </c>
-      <c r="W28" s="5" t="inlineStr">
+      <c r="W28" s="2" t="inlineStr"/>
+      <c r="X28" s="2" t="inlineStr"/>
+      <c r="Y28" s="2" t="inlineStr"/>
+      <c r="Z28" s="2" t="inlineStr"/>
+      <c r="AA28" s="2" t="inlineStr"/>
+      <c r="AB28" s="5" t="inlineStr">
         <is>
           <t>11MpXcVeE8r23ridBo2EJTqv7H9SnKWl3</t>
         </is>
       </c>
-      <c r="X28" s="5" t="inlineStr">
+      <c r="AC28" s="5" t="inlineStr">
         <is>
           <t>P060072.pdf</t>
         </is>
       </c>
-      <c r="Y28" s="5" t="inlineStr">
+      <c r="AD28" s="5" t="inlineStr">
         <is>
           <t>557493</t>
         </is>
       </c>
-      <c r="Z28" s="2" t="inlineStr"/>
+      <c r="AE28" s="2" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
@@ -4100,22 +4285,27 @@
           <t>0.007</t>
         </is>
       </c>
-      <c r="W29" s="5" t="inlineStr">
+      <c r="W29" s="2" t="inlineStr"/>
+      <c r="X29" s="2" t="inlineStr"/>
+      <c r="Y29" s="2" t="inlineStr"/>
+      <c r="Z29" s="2" t="inlineStr"/>
+      <c r="AA29" s="2" t="inlineStr"/>
+      <c r="AB29" s="5" t="inlineStr">
         <is>
           <t>1BUenYcQdiFfnWQeRHINp95V6eIfDfIUY</t>
         </is>
       </c>
-      <c r="X29" s="5" t="inlineStr">
+      <c r="AC29" s="5" t="inlineStr">
         <is>
           <t>P060092.pdf</t>
         </is>
       </c>
-      <c r="Y29" s="5" t="inlineStr">
+      <c r="AD29" s="5" t="inlineStr">
         <is>
           <t>551546</t>
         </is>
       </c>
-      <c r="Z29" s="2" t="inlineStr"/>
+      <c r="AE29" s="2" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
@@ -4224,22 +4414,27 @@
           <t>ND</t>
         </is>
       </c>
-      <c r="W30" s="5" t="inlineStr">
+      <c r="W30" s="2" t="inlineStr"/>
+      <c r="X30" s="2" t="inlineStr"/>
+      <c r="Y30" s="2" t="inlineStr"/>
+      <c r="Z30" s="2" t="inlineStr"/>
+      <c r="AA30" s="2" t="inlineStr"/>
+      <c r="AB30" s="5" t="inlineStr">
         <is>
           <t>1DNkgAKvnTQlkLOCGEtWCZQ8KVp-ai0AW</t>
         </is>
       </c>
-      <c r="X30" s="5" t="inlineStr">
+      <c r="AC30" s="5" t="inlineStr">
         <is>
           <t>P060112.pdf</t>
         </is>
       </c>
-      <c r="Y30" s="5" t="inlineStr">
+      <c r="AD30" s="5" t="inlineStr">
         <is>
           <t>543184</t>
         </is>
       </c>
-      <c r="Z30" s="2" t="inlineStr"/>
+      <c r="AE30" s="2" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
@@ -4348,22 +4543,27 @@
           <t>ND</t>
         </is>
       </c>
-      <c r="W31" s="5" t="inlineStr">
+      <c r="W31" s="2" t="inlineStr"/>
+      <c r="X31" s="2" t="inlineStr"/>
+      <c r="Y31" s="2" t="inlineStr"/>
+      <c r="Z31" s="2" t="inlineStr"/>
+      <c r="AA31" s="2" t="inlineStr"/>
+      <c r="AB31" s="5" t="inlineStr">
         <is>
           <t>1sNq4flkvkrjO7fT0OUTRPlL5Eb5fCYGX</t>
         </is>
       </c>
-      <c r="X31" s="5" t="inlineStr">
+      <c r="AC31" s="5" t="inlineStr">
         <is>
           <t>P060122.pdf</t>
         </is>
       </c>
-      <c r="Y31" s="5" t="inlineStr">
+      <c r="AD31" s="5" t="inlineStr">
         <is>
           <t>556221</t>
         </is>
       </c>
-      <c r="Z31" s="2" t="inlineStr"/>
+      <c r="AE31" s="2" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
@@ -4472,22 +4672,27 @@
           <t>ND</t>
         </is>
       </c>
-      <c r="W32" s="5" t="inlineStr">
+      <c r="W32" s="2" t="inlineStr"/>
+      <c r="X32" s="2" t="inlineStr"/>
+      <c r="Y32" s="2" t="inlineStr"/>
+      <c r="Z32" s="2" t="inlineStr"/>
+      <c r="AA32" s="2" t="inlineStr"/>
+      <c r="AB32" s="5" t="inlineStr">
         <is>
           <t>1dR9_VzZqRGMR6ywvFyCgsFcj1H7hL_YD</t>
         </is>
       </c>
-      <c r="X32" s="5" t="inlineStr">
+      <c r="AC32" s="5" t="inlineStr">
         <is>
           <t>P060132.pdf</t>
         </is>
       </c>
-      <c r="Y32" s="5" t="inlineStr">
+      <c r="AD32" s="5" t="inlineStr">
         <is>
           <t>543217</t>
         </is>
       </c>
-      <c r="Z32" s="2" t="inlineStr"/>
+      <c r="AE32" s="2" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
@@ -4600,22 +4805,27 @@
           <t>ND</t>
         </is>
       </c>
-      <c r="W33" s="5" t="inlineStr">
+      <c r="W33" s="2" t="inlineStr"/>
+      <c r="X33" s="2" t="inlineStr"/>
+      <c r="Y33" s="2" t="inlineStr"/>
+      <c r="Z33" s="2" t="inlineStr"/>
+      <c r="AA33" s="2" t="inlineStr"/>
+      <c r="AB33" s="5" t="inlineStr">
         <is>
           <t>1FnMN_MBQ1jhywZUFdKp2lhpx_yRMpbWW</t>
         </is>
       </c>
-      <c r="X33" s="5" t="inlineStr">
+      <c r="AC33" s="5" t="inlineStr">
         <is>
           <t>P060152 (1).pdf</t>
         </is>
       </c>
-      <c r="Y33" s="5" t="inlineStr">
+      <c r="AD33" s="5" t="inlineStr">
         <is>
           <t>515183</t>
         </is>
       </c>
-      <c r="Z33" s="2" t="inlineStr"/>
+      <c r="AE33" s="2" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
@@ -4724,22 +4934,27 @@
           <t>ND</t>
         </is>
       </c>
-      <c r="W34" s="5" t="inlineStr">
+      <c r="W34" s="2" t="inlineStr"/>
+      <c r="X34" s="2" t="inlineStr"/>
+      <c r="Y34" s="2" t="inlineStr"/>
+      <c r="Z34" s="2" t="inlineStr"/>
+      <c r="AA34" s="2" t="inlineStr"/>
+      <c r="AB34" s="5" t="inlineStr">
         <is>
           <t>1Vn3uRkNBWo4qpLNcLMVju7cUUjri0DIP</t>
         </is>
       </c>
-      <c r="X34" s="5" t="inlineStr">
+      <c r="AC34" s="5" t="inlineStr">
         <is>
           <t>P060172.pdf</t>
         </is>
       </c>
-      <c r="Y34" s="5" t="inlineStr">
+      <c r="AD34" s="5" t="inlineStr">
         <is>
           <t>538884</t>
         </is>
       </c>
-      <c r="Z34" s="2" t="inlineStr"/>
+      <c r="AE34" s="2" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
@@ -4848,22 +5063,27 @@
           <t>0.0013</t>
         </is>
       </c>
-      <c r="W35" s="5" t="inlineStr">
+      <c r="W35" s="2" t="inlineStr"/>
+      <c r="X35" s="2" t="inlineStr"/>
+      <c r="Y35" s="2" t="inlineStr"/>
+      <c r="Z35" s="2" t="inlineStr"/>
+      <c r="AA35" s="2" t="inlineStr"/>
+      <c r="AB35" s="5" t="inlineStr">
         <is>
           <t>1XgbYnZnUAmTSzVV0NsNmQwr2R5hRUs3e</t>
         </is>
       </c>
-      <c r="X35" s="5" t="inlineStr">
+      <c r="AC35" s="5" t="inlineStr">
         <is>
           <t>P060182.pdf</t>
         </is>
       </c>
-      <c r="Y35" s="5" t="inlineStr">
+      <c r="AD35" s="5" t="inlineStr">
         <is>
           <t>592468</t>
         </is>
       </c>
-      <c r="Z35" s="2" t="inlineStr">
+      <c r="AE35" s="2" t="inlineStr">
         <is>
           <t>9,11 credited to no laboratory</t>
         </is>
@@ -4980,22 +5200,27 @@
           <t>0.0166</t>
         </is>
       </c>
-      <c r="W36" s="5" t="inlineStr">
+      <c r="W36" s="2" t="inlineStr"/>
+      <c r="X36" s="2" t="inlineStr"/>
+      <c r="Y36" s="2" t="inlineStr"/>
+      <c r="Z36" s="2" t="inlineStr"/>
+      <c r="AA36" s="2" t="inlineStr"/>
+      <c r="AB36" s="5" t="inlineStr">
         <is>
           <t>1_3L98AHbmZJgVha3sMOsRBG6M6CN8-XU</t>
         </is>
       </c>
-      <c r="X36" s="5" t="inlineStr">
+      <c r="AC36" s="5" t="inlineStr">
         <is>
           <t>P060212 (1).pdf</t>
         </is>
       </c>
-      <c r="Y36" s="5" t="inlineStr">
+      <c r="AD36" s="5" t="inlineStr">
         <is>
           <t>522904</t>
         </is>
       </c>
-      <c r="Z36" s="2" t="inlineStr"/>
+      <c r="AE36" s="2" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
@@ -5104,22 +5329,47 @@
           <t>ND</t>
         </is>
       </c>
-      <c r="W37" s="5" t="inlineStr">
+      <c r="W37" s="2" t="inlineStr">
+        <is>
+          <t>ND</t>
+        </is>
+      </c>
+      <c r="X37" s="2" t="inlineStr">
+        <is>
+          <t>ND</t>
+        </is>
+      </c>
+      <c r="Y37" s="2" t="inlineStr">
+        <is>
+          <t>ND</t>
+        </is>
+      </c>
+      <c r="Z37" s="2" t="inlineStr">
+        <is>
+          <t>220-24-М/26 (11.09.2026)</t>
+        </is>
+      </c>
+      <c r="AA37" s="2" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="AB37" s="5" t="inlineStr">
         <is>
           <t>1Z0aBYrtZOqJF306LAOcHEj4ORK6ua1jc</t>
         </is>
       </c>
-      <c r="X37" s="5" t="inlineStr">
+      <c r="AC37" s="5" t="inlineStr">
         <is>
           <t>P060232.pdf</t>
         </is>
       </c>
-      <c r="Y37" s="5" t="inlineStr">
+      <c r="AD37" s="5" t="inlineStr">
         <is>
           <t>542158</t>
         </is>
       </c>
-      <c r="Z37" s="2" t="inlineStr"/>
+      <c r="AE37" s="2" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
@@ -5228,22 +5478,27 @@
           <t>ND</t>
         </is>
       </c>
-      <c r="W38" s="5" t="inlineStr">
+      <c r="W38" s="2" t="inlineStr"/>
+      <c r="X38" s="2" t="inlineStr"/>
+      <c r="Y38" s="2" t="inlineStr"/>
+      <c r="Z38" s="2" t="inlineStr"/>
+      <c r="AA38" s="2" t="inlineStr"/>
+      <c r="AB38" s="5" t="inlineStr">
         <is>
           <t>13_NX139vq60tP8JB9ht0FQmk5Ebg0KJU</t>
         </is>
       </c>
-      <c r="X38" s="5" t="inlineStr">
+      <c r="AC38" s="5" t="inlineStr">
         <is>
           <t>P060242 (1).pdf</t>
         </is>
       </c>
-      <c r="Y38" s="5" t="inlineStr">
+      <c r="AD38" s="5" t="inlineStr">
         <is>
           <t>524470</t>
         </is>
       </c>
-      <c r="Z38" s="2" t="inlineStr"/>
+      <c r="AE38" s="2" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
@@ -5352,22 +5607,27 @@
           <t>0.017</t>
         </is>
       </c>
-      <c r="W39" s="5" t="inlineStr">
+      <c r="W39" s="2" t="inlineStr"/>
+      <c r="X39" s="2" t="inlineStr"/>
+      <c r="Y39" s="2" t="inlineStr"/>
+      <c r="Z39" s="2" t="inlineStr"/>
+      <c r="AA39" s="2" t="inlineStr"/>
+      <c r="AB39" s="5" t="inlineStr">
         <is>
           <t>1m5V9BusVzXRnePzZwWZnquoACFtHyHhD</t>
         </is>
       </c>
-      <c r="X39" s="5" t="inlineStr">
+      <c r="AC39" s="5" t="inlineStr">
         <is>
           <t>P060282.pdf</t>
         </is>
       </c>
-      <c r="Y39" s="5" t="inlineStr">
+      <c r="AD39" s="5" t="inlineStr">
         <is>
           <t>537165</t>
         </is>
       </c>
-      <c r="Z39" s="2" t="inlineStr"/>
+      <c r="AE39" s="2" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
@@ -5476,22 +5736,27 @@
           <t>0.0155</t>
         </is>
       </c>
-      <c r="W40" s="5" t="inlineStr">
+      <c r="W40" s="2" t="inlineStr"/>
+      <c r="X40" s="2" t="inlineStr"/>
+      <c r="Y40" s="2" t="inlineStr"/>
+      <c r="Z40" s="2" t="inlineStr"/>
+      <c r="AA40" s="2" t="inlineStr"/>
+      <c r="AB40" s="5" t="inlineStr">
         <is>
           <t>1YYNMjGRChveckb4BtIiyaHq9ywgA4cBU</t>
         </is>
       </c>
-      <c r="X40" s="5" t="inlineStr">
+      <c r="AC40" s="5" t="inlineStr">
         <is>
           <t>P060322.pdf</t>
         </is>
       </c>
-      <c r="Y40" s="5" t="inlineStr">
+      <c r="AD40" s="5" t="inlineStr">
         <is>
           <t>558402</t>
         </is>
       </c>
-      <c r="Z40" s="2" t="inlineStr"/>
+      <c r="AE40" s="2" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
@@ -5600,22 +5865,27 @@
           <t>0.002</t>
         </is>
       </c>
-      <c r="W41" s="5" t="inlineStr">
+      <c r="W41" s="2" t="inlineStr"/>
+      <c r="X41" s="2" t="inlineStr"/>
+      <c r="Y41" s="2" t="inlineStr"/>
+      <c r="Z41" s="2" t="inlineStr"/>
+      <c r="AA41" s="2" t="inlineStr"/>
+      <c r="AB41" s="5" t="inlineStr">
         <is>
           <t>1LCLmwHYZ2i15KONPddkbjaOy_SQNmbKR</t>
         </is>
       </c>
-      <c r="X41" s="5" t="inlineStr">
+      <c r="AC41" s="5" t="inlineStr">
         <is>
           <t>P060352 (1).pdf</t>
         </is>
       </c>
-      <c r="Y41" s="5" t="inlineStr">
+      <c r="AD41" s="5" t="inlineStr">
         <is>
           <t>539353</t>
         </is>
       </c>
-      <c r="Z41" s="2" t="inlineStr"/>
+      <c r="AE41" s="2" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
@@ -5728,22 +5998,27 @@
           <t>0.002</t>
         </is>
       </c>
-      <c r="W42" s="5" t="inlineStr">
+      <c r="W42" s="2" t="inlineStr"/>
+      <c r="X42" s="2" t="inlineStr"/>
+      <c r="Y42" s="2" t="inlineStr"/>
+      <c r="Z42" s="2" t="inlineStr"/>
+      <c r="AA42" s="2" t="inlineStr"/>
+      <c r="AB42" s="5" t="inlineStr">
         <is>
           <t>1Dq-Bo-EMu6T3sFZztVxUxzh4ZwoARlFC</t>
         </is>
       </c>
-      <c r="X42" s="5" t="inlineStr">
+      <c r="AC42" s="5" t="inlineStr">
         <is>
           <t>P060362.pdf</t>
         </is>
       </c>
-      <c r="Y42" s="5" t="inlineStr">
+      <c r="AD42" s="5" t="inlineStr">
         <is>
           <t>545349</t>
         </is>
       </c>
-      <c r="Z42" s="2" t="inlineStr">
+      <c r="AE42" s="2" t="inlineStr">
         <is>
           <t>foreign matter (7) credited to CNP, not in-house</t>
         </is>
@@ -5860,22 +6135,27 @@
           <t>0.001</t>
         </is>
       </c>
-      <c r="W43" s="5" t="inlineStr">
+      <c r="W43" s="2" t="inlineStr"/>
+      <c r="X43" s="2" t="inlineStr"/>
+      <c r="Y43" s="2" t="inlineStr"/>
+      <c r="Z43" s="2" t="inlineStr"/>
+      <c r="AA43" s="2" t="inlineStr"/>
+      <c r="AB43" s="5" t="inlineStr">
         <is>
           <t>1wV5kgsgWcFxdiivC3aIca0pFEL0KHYbn</t>
         </is>
       </c>
-      <c r="X43" s="5" t="inlineStr">
+      <c r="AC43" s="5" t="inlineStr">
         <is>
           <t>P060372.pdf</t>
         </is>
       </c>
-      <c r="Y43" s="5" t="inlineStr">
+      <c r="AD43" s="5" t="inlineStr">
         <is>
           <t>599453</t>
         </is>
       </c>
-      <c r="Z43" s="2" t="inlineStr"/>
+      <c r="AE43" s="2" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
@@ -5984,22 +6264,27 @@
           <t>0.004</t>
         </is>
       </c>
-      <c r="W44" s="5" t="inlineStr">
+      <c r="W44" s="2" t="inlineStr"/>
+      <c r="X44" s="2" t="inlineStr"/>
+      <c r="Y44" s="2" t="inlineStr"/>
+      <c r="Z44" s="2" t="inlineStr"/>
+      <c r="AA44" s="2" t="inlineStr"/>
+      <c r="AB44" s="5" t="inlineStr">
         <is>
           <t>1gzWGarZb0fgyJG1PNDfxRDpu6RP4RJ_7</t>
         </is>
       </c>
-      <c r="X44" s="5" t="inlineStr">
+      <c r="AC44" s="5" t="inlineStr">
         <is>
           <t>P060382 (1).pdf</t>
         </is>
       </c>
-      <c r="Y44" s="5" t="inlineStr">
+      <c r="AD44" s="5" t="inlineStr">
         <is>
           <t>544029</t>
         </is>
       </c>
-      <c r="Z44" s="2" t="inlineStr"/>
+      <c r="AE44" s="2" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
@@ -6108,22 +6393,27 @@
           <t>0.015</t>
         </is>
       </c>
-      <c r="W45" s="5" t="inlineStr">
+      <c r="W45" s="2" t="inlineStr"/>
+      <c r="X45" s="2" t="inlineStr"/>
+      <c r="Y45" s="2" t="inlineStr"/>
+      <c r="Z45" s="2" t="inlineStr"/>
+      <c r="AA45" s="2" t="inlineStr"/>
+      <c r="AB45" s="5" t="inlineStr">
         <is>
           <t>131nSAU0wesNOCQGdpyuCYTcsqr283vlD</t>
         </is>
       </c>
-      <c r="X45" s="5" t="inlineStr">
+      <c r="AC45" s="5" t="inlineStr">
         <is>
           <t>P060402 (1).pdf</t>
         </is>
       </c>
-      <c r="Y45" s="5" t="inlineStr">
+      <c r="AD45" s="5" t="inlineStr">
         <is>
           <t>550537</t>
         </is>
       </c>
-      <c r="Z45" s="2" t="inlineStr">
+      <c r="AE45" s="2" t="inlineStr">
         <is>
           <t>no iCoA row; 1,2,7,8 credited to CNP</t>
         </is>
@@ -6240,22 +6530,27 @@
           <t>0.042</t>
         </is>
       </c>
-      <c r="W46" s="5" t="inlineStr">
+      <c r="W46" s="2" t="inlineStr"/>
+      <c r="X46" s="2" t="inlineStr"/>
+      <c r="Y46" s="2" t="inlineStr"/>
+      <c r="Z46" s="2" t="inlineStr"/>
+      <c r="AA46" s="2" t="inlineStr"/>
+      <c r="AB46" s="5" t="inlineStr">
         <is>
           <t>1QXRoZx2T6_-46KBIja-TwV-sRAS7erYU</t>
         </is>
       </c>
-      <c r="X46" s="5" t="inlineStr">
+      <c r="AC46" s="5" t="inlineStr">
         <is>
           <t>P060412.pdf</t>
         </is>
       </c>
-      <c r="Y46" s="5" t="inlineStr">
+      <c r="AD46" s="5" t="inlineStr">
         <is>
           <t>577676</t>
         </is>
       </c>
-      <c r="Z46" s="2" t="inlineStr">
+      <c r="AE46" s="2" t="inlineStr">
         <is>
           <t>no iCoA row; 1,2,7,8 credited to CNP</t>
         </is>
@@ -6372,29 +6667,34 @@
           <t>0.045</t>
         </is>
       </c>
-      <c r="W47" s="5" t="inlineStr">
+      <c r="W47" s="2" t="inlineStr"/>
+      <c r="X47" s="2" t="inlineStr"/>
+      <c r="Y47" s="2" t="inlineStr"/>
+      <c r="Z47" s="2" t="inlineStr"/>
+      <c r="AA47" s="2" t="inlineStr"/>
+      <c r="AB47" s="5" t="inlineStr">
         <is>
           <t>1w2GtdmjLog-xSZdeSy-r0M-51JLfJ391</t>
         </is>
       </c>
-      <c r="X47" s="5" t="inlineStr">
+      <c r="AC47" s="5" t="inlineStr">
         <is>
           <t>P060422.pdf</t>
         </is>
       </c>
-      <c r="Y47" s="5" t="inlineStr">
+      <c r="AD47" s="5" t="inlineStr">
         <is>
           <t>601712</t>
         </is>
       </c>
-      <c r="Z47" s="2" t="inlineStr">
+      <c r="AE47" s="2" t="inlineStr">
         <is>
           <t>9,11 credited to no laboratory</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:Z47"/>
+  <autoFilter ref="A1:AE47"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>